<commit_message>
Final prose draft, still needs other files
</commit_message>
<xml_diff>
--- a/Test_Data/analysis/data_v2/fig_general_comparison.xlsx
+++ b/Test_Data/analysis/data_v2/fig_general_comparison.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Documents\Thesis\thesis\Test_Data\analysis\data_v2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC868373-6441-42DC-8CE4-B0B685575A9F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0CBD056-7201-48EF-9074-7213DD9FCC41}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="38280" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="332" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="332" uniqueCount="33">
   <si>
     <t>series</t>
   </si>
@@ -114,6 +114,15 @@
   </si>
   <si>
     <t>C (10 m)</t>
+  </si>
+  <si>
+    <t>5G Round1</t>
+  </si>
+  <si>
+    <t>5G Round2</t>
+  </si>
+  <si>
+    <t>5G Round3</t>
   </si>
 </sst>
 </file>
@@ -351,7 +360,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>5G_1</c:v>
+                  <c:v>5G Round1</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -466,7 +475,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>5G_2</c:v>
+                  <c:v>5G Round2</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -599,7 +608,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>5G_3</c:v>
+                  <c:v>5G Round3</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -1064,7 +1073,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>5G_1</c:v>
+                  <c:v>5G Round1</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -1179,7 +1188,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>5G_2</c:v>
+                  <c:v>5G Round2</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -1312,7 +1321,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>5G_3</c:v>
+                  <c:v>5G Round3</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -1777,7 +1786,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>5G_1</c:v>
+                  <c:v>5G Round1</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -1892,7 +1901,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>5G_2</c:v>
+                  <c:v>5G Round2</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -2025,7 +2034,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>5G_3</c:v>
+                  <c:v>5G Round3</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -2490,7 +2499,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>5G_1</c:v>
+                  <c:v>5G Round1</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -2605,7 +2614,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>5G_2</c:v>
+                  <c:v>5G Round2</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -2738,7 +2747,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>5G_3</c:v>
+                  <c:v>5G Round3</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -5260,13 +5269,13 @@
         <v>12</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>17</v>
+        <v>30</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>18</v>
+        <v>31</v>
       </c>
       <c r="K1" s="3" t="s">
-        <v>19</v>
+        <v>32</v>
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
@@ -5452,13 +5461,13 @@
         <v>12</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>17</v>
+        <v>30</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>18</v>
+        <v>31</v>
       </c>
       <c r="K1" s="3" t="s">
-        <v>19</v>
+        <v>32</v>
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
@@ -5644,13 +5653,13 @@
         <v>12</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>17</v>
+        <v>30</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>18</v>
+        <v>31</v>
       </c>
       <c r="K1" s="3" t="s">
-        <v>19</v>
+        <v>32</v>
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
@@ -5836,13 +5845,13 @@
         <v>12</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>17</v>
+        <v>30</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>18</v>
+        <v>31</v>
       </c>
       <c r="K1" s="3" t="s">
-        <v>19</v>
+        <v>32</v>
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">

</xml_diff>